<commit_message>
Polished README file and sprint 1 notes published.
</commit_message>
<xml_diff>
--- a/scrum/burndown_chart.xlsx
+++ b/scrum/burndown_chart.xlsx
@@ -417,14 +417,17 @@
       <c r="A2" t="str">
         <v>Planned</v>
       </c>
+      <c r="B2" t="str">
+        <v>32</v>
+      </c>
       <c r="C2" t="str">
-        <v>75</v>
+        <v>6</v>
       </c>
       <c r="D2" t="str">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="E2" t="str">
-        <v>40</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -432,13 +435,13 @@
         <v>Actual</v>
       </c>
       <c r="C3" t="str">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="D3" t="str">
-        <v>45</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>40</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -446,10 +449,10 @@
         <v>Ideal</v>
       </c>
       <c r="C4" t="str">
-        <v>175</v>
+        <v>26</v>
       </c>
       <c r="D4" t="str">
-        <v>140</v>
+        <v>5</v>
       </c>
       <c r="E4" t="str">
         <v>0</v>
@@ -460,13 +463,13 @@
         <v>Remaining</v>
       </c>
       <c r="B5" t="str">
-        <v>250</v>
+        <v>32</v>
       </c>
       <c r="C5" t="str">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="D5" t="str">
-        <v>155</v>
+        <v/>
       </c>
       <c r="E5" t="str">
         <v>0</v>

</xml_diff>

<commit_message>
Scrum notes compiled and readme updated to complete sprint 2.
</commit_message>
<xml_diff>
--- a/scrum/burndown_chart.xlsx
+++ b/scrum/burndown_chart.xlsx
@@ -438,7 +438,7 @@
         <v>6</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>21</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -469,7 +469,7 @@
         <v>26</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="E5" t="str">
         <v>0</v>

</xml_diff>

<commit_message>
Fixed scrum notes to follow structure, polished readme, added coverage report, added burndown chart, and removed unnecessary files.
</commit_message>
<xml_diff>
--- a/scrum/burndown_chart.xlsx
+++ b/scrum/burndown_chart.xlsx
@@ -427,7 +427,7 @@
         <v>21</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -441,18 +441,21 @@
         <v>21</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>Ideal</v>
       </c>
+      <c r="B4" t="str">
+        <v>32</v>
+      </c>
       <c r="C4" t="str">
-        <v>26</v>
+        <v>21.33</v>
       </c>
       <c r="D4" t="str">
-        <v>5</v>
+        <v>10.66</v>
       </c>
       <c r="E4" t="str">
         <v>0</v>

</xml_diff>